<commit_message>
Update final dataset and Orange workflow
Updated student dataset, finalized Orange workflow configuration, and synchronized dashboard data.
</commit_message>
<xml_diff>
--- a/student_risk_dataset.xlsx
+++ b/student_risk_dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\da2\Desktop\Masoud Projects\DA\2026\2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tamim/Desktop/واجبات الفصل الصيفي/it475/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D61068EA-6CC2-4E4A-BC79-88C85BEB4A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EC9C402-F202-0144-8F6D-D1B6A60EF387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="23260" windowHeight="12580" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Student Data" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="159">
   <si>
     <t>SPSS Educator Dashboard — Student Risk Overview</t>
   </si>
@@ -124,9 +124,6 @@
     <t>GREEN - Satisfactory</t>
   </si>
   <si>
-    <t>Weekly Risk Trend (illustrative sample — replace with real weekly snapshot counts)</t>
-  </si>
-  <si>
     <t>Week</t>
   </si>
   <si>
@@ -220,246 +217,123 @@
     <t>STU1001</t>
   </si>
   <si>
-    <t>Emma Smith</t>
-  </si>
-  <si>
     <t>STU1002</t>
   </si>
   <si>
-    <t>Liam Johnson</t>
-  </si>
-  <si>
     <t>STU1003</t>
   </si>
   <si>
-    <t>Olivia Williams</t>
-  </si>
-  <si>
     <t>STU1004</t>
   </si>
   <si>
-    <t>Noah Brown</t>
-  </si>
-  <si>
     <t>STU1005</t>
   </si>
   <si>
-    <t>Ava Jones</t>
-  </si>
-  <si>
     <t>STU1006</t>
   </si>
   <si>
-    <t>Ethan Garcia</t>
-  </si>
-  <si>
     <t>STU1007</t>
   </si>
   <si>
-    <t>Sophia Miller</t>
-  </si>
-  <si>
     <t>STU1008</t>
   </si>
   <si>
-    <t>Mason Davis</t>
-  </si>
-  <si>
     <t>STU1009</t>
   </si>
   <si>
-    <t>Isabella Rodriguez</t>
-  </si>
-  <si>
     <t>STU1010</t>
   </si>
   <si>
-    <t>Lucas Martinez</t>
-  </si>
-  <si>
     <t>STU1011</t>
   </si>
   <si>
-    <t>Mia Hernandez</t>
-  </si>
-  <si>
     <t>STU1012</t>
   </si>
   <si>
-    <t>James Lopez</t>
-  </si>
-  <si>
     <t>STU1013</t>
   </si>
   <si>
-    <t>Amelia Gonzalez</t>
-  </si>
-  <si>
     <t>STU1014</t>
   </si>
   <si>
-    <t>Benjamin Wilson</t>
-  </si>
-  <si>
     <t>STU1015</t>
   </si>
   <si>
-    <t>Charlotte Anderson</t>
-  </si>
-  <si>
     <t>STU1016</t>
   </si>
   <si>
-    <t>Elijah Thomas</t>
-  </si>
-  <si>
     <t>STU1017</t>
   </si>
   <si>
-    <t>Harper Taylor</t>
-  </si>
-  <si>
     <t>STU1018</t>
   </si>
   <si>
-    <t>Logan Moore</t>
-  </si>
-  <si>
     <t>STU1019</t>
   </si>
   <si>
-    <t>Evelyn Jackson</t>
-  </si>
-  <si>
     <t>STU1020</t>
   </si>
   <si>
-    <t>Alexander Martin</t>
-  </si>
-  <si>
     <t>STU1021</t>
   </si>
   <si>
-    <t>Abigail Lee</t>
-  </si>
-  <si>
     <t>STU1022</t>
   </si>
   <si>
-    <t>Michael Perez</t>
-  </si>
-  <si>
     <t>STU1023</t>
   </si>
   <si>
-    <t>Emily Thompson</t>
-  </si>
-  <si>
     <t>STU1024</t>
   </si>
   <si>
-    <t>Daniel White</t>
-  </si>
-  <si>
     <t>STU1025</t>
   </si>
   <si>
-    <t>Ella Harris</t>
-  </si>
-  <si>
     <t>STU1026</t>
   </si>
   <si>
-    <t>Henry Sanchez</t>
-  </si>
-  <si>
     <t>STU1027</t>
   </si>
   <si>
-    <t>Scarlett Clark</t>
-  </si>
-  <si>
     <t>STU1028</t>
   </si>
   <si>
-    <t>Jackson Ramirez</t>
-  </si>
-  <si>
     <t>STU1029</t>
   </si>
   <si>
-    <t>Grace Lewis</t>
-  </si>
-  <si>
     <t>STU1030</t>
   </si>
   <si>
-    <t>Sebastian Robinson</t>
-  </si>
-  <si>
     <t>STU1031</t>
   </si>
   <si>
-    <t>Chloe Walker</t>
-  </si>
-  <si>
     <t>STU1032</t>
   </si>
   <si>
-    <t>Aiden Young</t>
-  </si>
-  <si>
     <t>STU1033</t>
   </si>
   <si>
-    <t>Victoria Allen</t>
-  </si>
-  <si>
     <t>STU1034</t>
   </si>
   <si>
-    <t>Matthew King</t>
-  </si>
-  <si>
     <t>STU1035</t>
   </si>
   <si>
-    <t>Riley Wright</t>
-  </si>
-  <si>
     <t>STU1036</t>
   </si>
   <si>
-    <t>Samuel Scott</t>
-  </si>
-  <si>
     <t>STU1037</t>
   </si>
   <si>
-    <t>Aria Torres</t>
-  </si>
-  <si>
     <t>STU1038</t>
   </si>
   <si>
-    <t>David Nguyen</t>
-  </si>
-  <si>
     <t>STU1039</t>
   </si>
   <si>
-    <t>Lily Hill</t>
-  </si>
-  <si>
     <t>STU1040</t>
   </si>
   <si>
-    <t>Joseph Flores</t>
-  </si>
-  <si>
-    <t>Threshold Line Helpers -&gt;</t>
-  </si>
-  <si>
     <t>SPSS Sample Dataset - Placeholder Data</t>
   </si>
   <si>
@@ -472,12 +346,6 @@
     <t>Structure:</t>
   </si>
   <si>
-    <t>- 40 fictional students, evenly split across all 4 risk categories (10 each):</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  RED (fails both), YELLOW (fails academic only or attendance only - 20 total), GREEN (passes both)</t>
-  </si>
-  <si>
     <t>Thresholds used (as defined in the project):</t>
   </si>
   <si>
@@ -518,6 +386,135 @@
   </si>
   <si>
     <t>Column1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weekly Risk Trend </t>
+  </si>
+  <si>
+    <t>Ahmed Mohammed</t>
+  </si>
+  <si>
+    <t>Khalid Abdullah</t>
+  </si>
+  <si>
+    <t>Saud Ibrahim</t>
+  </si>
+  <si>
+    <t>Mohammed Ali</t>
+  </si>
+  <si>
+    <t>Fahad Saleh</t>
+  </si>
+  <si>
+    <t>Abdullah Hassan</t>
+  </si>
+  <si>
+    <t>Omar Khalid</t>
+  </si>
+  <si>
+    <t>Yousef Ahmed</t>
+  </si>
+  <si>
+    <t>Nasser Saad</t>
+  </si>
+  <si>
+    <t>Turki Mohammed</t>
+  </si>
+  <si>
+    <t>Abdulrahman Ali</t>
+  </si>
+  <si>
+    <t>Sultan Fahad</t>
+  </si>
+  <si>
+    <t>Majed Abdullah</t>
+  </si>
+  <si>
+    <t>Badr Ibrahim</t>
+  </si>
+  <si>
+    <t>Ziyad Hassan</t>
+  </si>
+  <si>
+    <t>Waleed Saleh</t>
+  </si>
+  <si>
+    <t>Sami Khalid</t>
+  </si>
+  <si>
+    <t>Faisal Mohammed</t>
+  </si>
+  <si>
+    <t>Sarah Mohammed</t>
+  </si>
+  <si>
+    <t>Nora Khalid</t>
+  </si>
+  <si>
+    <t>Reem Abdullah</t>
+  </si>
+  <si>
+    <t>Huda Ahmed</t>
+  </si>
+  <si>
+    <t>Lina Saleh</t>
+  </si>
+  <si>
+    <t>Maha Ibrahim</t>
+  </si>
+  <si>
+    <t>Amal Hassan</t>
+  </si>
+  <si>
+    <t>Dana Mohammed</t>
+  </si>
+  <si>
+    <t>Joud Khalid</t>
+  </si>
+  <si>
+    <t>Lama Abdullah</t>
+  </si>
+  <si>
+    <t>Shahad Ahmed</t>
+  </si>
+  <si>
+    <t>Maryam Saleh</t>
+  </si>
+  <si>
+    <t>Rana Ibrahim</t>
+  </si>
+  <si>
+    <t>Abeer Hassan</t>
+  </si>
+  <si>
+    <t>Haifa Mohammed</t>
+  </si>
+  <si>
+    <t>Mona Khalid</t>
+  </si>
+  <si>
+    <t>Noor Abdullah</t>
+  </si>
+  <si>
+    <t>Arwa Ahmed</t>
+  </si>
+  <si>
+    <t>Layan Saleh</t>
+  </si>
+  <si>
+    <t>Ghada Ibrahim</t>
+  </si>
+  <si>
+    <t>Rawan Ahmed</t>
+  </si>
+  <si>
+    <t>Haneen Abdullah</t>
+  </si>
+  <si>
+    <t>- 40 fictional students distributed across 3 risk categories:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  RED (10 students), YELLOW (20 students), GREEN (10 students)</t>
   </si>
 </sst>
 </file>
@@ -529,7 +526,7 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.0\%"/>
   </numFmts>
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -542,148 +539,148 @@
       <sz val="18"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FFA6A6A6"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF595959"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FFA6A6A6"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="26"/>
       <color rgb="FF1F3864"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="26"/>
       <color rgb="FFC00000"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="26"/>
       <color rgb="FFBF8F00"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="26"/>
       <color rgb="FF548235"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="26"/>
       <color rgb="FF2F5597"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF808080"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FF595959"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF1F3864"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF1F3864"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFC00000"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFBF8F00"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF548235"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FFC00000"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FFBF8F00"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF548235"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -691,30 +688,42 @@
       <sz val="9"/>
       <color rgb="FFA6A6A6"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FFD9D9D9"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="8"/>
       <color rgb="FFA6A6A6"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -811,7 +820,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -860,23 +869,8 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="8" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -899,9 +893,27 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="1" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="8" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="عادي" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="20">
     <dxf>
@@ -945,24 +957,6 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FFA6A6A6"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-        <scheme val="none"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -1266,6 +1260,24 @@
       </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FFA6A6A6"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1350,7 +1362,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="ar-SA"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -1799,7 +1811,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="ar-SA"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -2167,7 +2179,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="ar-SA"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -2279,34 +2291,34 @@
               <c:strCache>
                 <c:ptCount val="31"/>
                 <c:pt idx="3">
-                  <c:v>92.2%</c:v>
+                  <c:v>92٫2%</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>84.2%</c:v>
+                  <c:v>84٫2%</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>81.1%</c:v>
+                  <c:v>81٫1%</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>84.3%</c:v>
+                  <c:v>84٫3%</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>78.1%</c:v>
+                  <c:v>78٫1%</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>86.0%</c:v>
+                  <c:v>86٫0%</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>98.4%</c:v>
+                  <c:v>98٫4%</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>87.2%</c:v>
+                  <c:v>87٫2%</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>81.5%</c:v>
+                  <c:v>81٫5%</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>79.8%</c:v>
+                  <c:v>79٫8%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2327,7 +2339,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3" formatCode="0.0">
-                  <c:v>84.666666666666671</c:v>
+                  <c:v>84.7</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2336,7 +2348,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6" formatCode="0.0">
-                  <c:v>79.666666666666671</c:v>
+                  <c:v>79.7</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -2345,7 +2357,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9" formatCode="0.0">
-                  <c:v>86.333333333333329</c:v>
+                  <c:v>86.3</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -2363,10 +2375,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15" formatCode="0.0">
-                  <c:v>90.666666666666671</c:v>
+                  <c:v>90.7</c:v>
                 </c:pt>
                 <c:pt idx="16" formatCode="0.0">
-                  <c:v>84.666666666666671</c:v>
+                  <c:v>84.7</c:v>
                 </c:pt>
                 <c:pt idx="17">
                   <c:v>0</c:v>
@@ -2381,7 +2393,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="21" formatCode="0.0">
-                  <c:v>76.333333333333329</c:v>
+                  <c:v>76.3</c:v>
                 </c:pt>
                 <c:pt idx="22" formatCode="0.0">
                   <c:v>76</c:v>
@@ -2396,10 +2408,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="26" formatCode="0.0">
-                  <c:v>78.666666666666671</c:v>
+                  <c:v>78.7</c:v>
                 </c:pt>
                 <c:pt idx="27" formatCode="0.0">
-                  <c:v>77.333333333333329</c:v>
+                  <c:v>77.3</c:v>
                 </c:pt>
                 <c:pt idx="28">
                   <c:v>0</c:v>
@@ -2408,7 +2420,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="30" formatCode="0.0">
-                  <c:v>85.333333333333329</c:v>
+                  <c:v>85.3</c:v>
                 </c:pt>
                 <c:pt idx="31">
                   <c:v>0</c:v>
@@ -2515,64 +2527,64 @@
               <c:strCache>
                 <c:ptCount val="38"/>
                 <c:pt idx="2">
-                  <c:v>82.4%</c:v>
+                  <c:v>82٫4%</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>73.6%</c:v>
+                  <c:v>73٫6%</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>56.7%</c:v>
+                  <c:v>56٫7%</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>90.0%</c:v>
+                  <c:v>90٫0%</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>69.7%</c:v>
+                  <c:v>69٫7%</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>51.6%</c:v>
+                  <c:v>51٫6%</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>59.5%</c:v>
+                  <c:v>59٫5%</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>79.1%</c:v>
+                  <c:v>79٫1%</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>92.4%</c:v>
+                  <c:v>92٫4%</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>65.1%</c:v>
+                  <c:v>65٫1%</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>84.5%</c:v>
+                  <c:v>84٫5%</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>73.3%</c:v>
+                  <c:v>73٫3%</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>68.0%</c:v>
+                  <c:v>68٫0%</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>70.9%</c:v>
+                  <c:v>70٫9%</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>80.4%</c:v>
+                  <c:v>80٫4%</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>97.0%</c:v>
+                  <c:v>97٫0%</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>72.3%</c:v>
+                  <c:v>72٫3%</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>88.9%</c:v>
+                  <c:v>88٫9%</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>76.2%</c:v>
+                  <c:v>76٫2%</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>95.9%</c:v>
+                  <c:v>95٫9%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2590,22 +2602,22 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2" formatCode="0.0">
-                  <c:v>50.333333333333336</c:v>
+                  <c:v>50.3</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4" formatCode="0.0">
-                  <c:v>72.333333333333329</c:v>
+                  <c:v>72.3</c:v>
                 </c:pt>
                 <c:pt idx="5" formatCode="0.0">
-                  <c:v>75.666666666666671</c:v>
+                  <c:v>75.7</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7" formatCode="0.0">
-                  <c:v>49.666666666666664</c:v>
+                  <c:v>49.7</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -2614,16 +2626,16 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10" formatCode="0.0">
-                  <c:v>73.333333333333329</c:v>
+                  <c:v>73.3</c:v>
                 </c:pt>
                 <c:pt idx="11" formatCode="0.0">
-                  <c:v>81.666666666666671</c:v>
+                  <c:v>81.7</c:v>
                 </c:pt>
                 <c:pt idx="12" formatCode="0.0">
-                  <c:v>82.333333333333329</c:v>
+                  <c:v>82.3</c:v>
                 </c:pt>
                 <c:pt idx="13" formatCode="0.0">
-                  <c:v>48.666666666666664</c:v>
+                  <c:v>48.7</c:v>
                 </c:pt>
                 <c:pt idx="14" formatCode="0.0">
                   <c:v>54</c:v>
@@ -2635,16 +2647,16 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="17" formatCode="0.0">
-                  <c:v>67.333333333333329</c:v>
+                  <c:v>67.3</c:v>
                 </c:pt>
                 <c:pt idx="18" formatCode="0.0">
-                  <c:v>51.333333333333336</c:v>
+                  <c:v>51.3</c:v>
                 </c:pt>
                 <c:pt idx="19" formatCode="0.0">
                   <c:v>87</c:v>
                 </c:pt>
                 <c:pt idx="20" formatCode="0.0">
-                  <c:v>74.666666666666671</c:v>
+                  <c:v>74.7</c:v>
                 </c:pt>
                 <c:pt idx="21">
                   <c:v>0</c:v>
@@ -2653,10 +2665,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="23" formatCode="0.0">
-                  <c:v>77.333333333333329</c:v>
+                  <c:v>77.3</c:v>
                 </c:pt>
                 <c:pt idx="24" formatCode="0.0">
-                  <c:v>54.666666666666664</c:v>
+                  <c:v>54.7</c:v>
                 </c:pt>
                 <c:pt idx="25" formatCode="0.0">
                   <c:v>51</c:v>
@@ -2677,7 +2689,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="31" formatCode="0.0">
-                  <c:v>85.333333333333329</c:v>
+                  <c:v>85.3</c:v>
                 </c:pt>
                 <c:pt idx="32">
                   <c:v>0</c:v>
@@ -2692,10 +2704,10 @@
                   <c:v>44</c:v>
                 </c:pt>
                 <c:pt idx="36" formatCode="0.0">
-                  <c:v>50.666666666666664</c:v>
+                  <c:v>50.7</c:v>
                 </c:pt>
                 <c:pt idx="37" formatCode="0.0">
-                  <c:v>43.333333333333336</c:v>
+                  <c:v>43.3</c:v>
                 </c:pt>
                 <c:pt idx="38">
                   <c:v>0</c:v>
@@ -2781,34 +2793,34 @@
               <c:strCache>
                 <c:ptCount val="40"/>
                 <c:pt idx="0">
-                  <c:v>56.3%</c:v>
+                  <c:v>56٫3%</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>62.9%</c:v>
+                  <c:v>62٫9%</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>53.9%</c:v>
+                  <c:v>53٫9%</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>52.1%</c:v>
+                  <c:v>52٫1%</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>68.4%</c:v>
+                  <c:v>68٫4%</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>67.1%</c:v>
+                  <c:v>67٫1%</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>59.0%</c:v>
+                  <c:v>59٫0%</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>55.9%</c:v>
+                  <c:v>55٫9%</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>55.7%</c:v>
+                  <c:v>55٫7%</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>62.9%</c:v>
+                  <c:v>62٫9%</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2820,10 +2832,10 @@
                 <c:formatCode>0.0</c:formatCode>
                 <c:ptCount val="42"/>
                 <c:pt idx="0">
-                  <c:v>48.666666666666664</c:v>
+                  <c:v>48.7</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>47.666666666666664</c:v>
+                  <c:v>47.7</c:v>
                 </c:pt>
                 <c:pt idx="2" formatCode="General">
                   <c:v>0</c:v>
@@ -2844,7 +2856,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>50.666666666666664</c:v>
+                  <c:v>50.7</c:v>
                 </c:pt>
                 <c:pt idx="9" formatCode="General">
                   <c:v>0</c:v>
@@ -2907,7 +2919,7 @@
                   <c:v>44</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>46.333333333333336</c:v>
+                  <c:v>46.3</c:v>
                 </c:pt>
                 <c:pt idx="30" formatCode="General">
                   <c:v>0</c:v>
@@ -2919,7 +2931,7 @@
                   <c:v>52</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>52.666666666666664</c:v>
+                  <c:v>52.7</c:v>
                 </c:pt>
                 <c:pt idx="34">
                   <c:v>46</c:v>
@@ -2934,7 +2946,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>44.333333333333336</c:v>
+                  <c:v>44.3</c:v>
                 </c:pt>
                 <c:pt idx="39">
                   <c:v>49</c:v>
@@ -3362,7 +3374,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="ar-SA"/>
   <c:roundedCorners val="0"/>
   <c:style val="2"/>
   <c:chart>
@@ -3387,7 +3399,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>Weekly Risk Trend (Illustrative Sample)</a:t>
+              <a:t>Weekly Risk Trend </a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -4161,44 +4173,44 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0471C492-2B49-4E34-8633-039E40797257}" name="Table1" displayName="Table1" ref="A1:U41" totalsRowShown="0" headerRowDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{0471C492-2B49-4E34-8633-039E40797257}" name="Table1" displayName="Table1" ref="A1:U41" totalsRowShown="0" headerRowDxfId="19">
   <autoFilter ref="A1:U41" xr:uid="{0471C492-2B49-4E34-8633-039E40797257}"/>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{C609D982-0FF1-4636-BE62-7A4277A17704}" name="Student ID" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{C4856892-C900-4B37-B98B-1E5F5CFE7DD4}" name="Name" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{1C8D9A67-14AE-4290-BC5D-7700B9C99E66}" name="Test 1" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{E06F4E46-70D3-4942-802E-F8E009985D05}" name="Test 2" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{3612BB37-905B-41F3-885C-8BE9593A4B4E}" name="Test 3" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{8088215E-C1E3-4276-8E6B-CB557AF551FA}" name="Average" dataDxfId="14">
-      <calculatedColumnFormula>AVERAGE(C2:E2)</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{C609D982-0FF1-4636-BE62-7A4277A17704}" name="Student ID" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{C4856892-C900-4B37-B98B-1E5F5CFE7DD4}" name="Name" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{1C8D9A67-14AE-4290-BC5D-7700B9C99E66}" name="Test 1" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{E06F4E46-70D3-4942-802E-F8E009985D05}" name="Test 2" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{3612BB37-905B-41F3-885C-8BE9593A4B4E}" name="Test 3" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{8088215E-C1E3-4276-8E6B-CB557AF551FA}" name="Average" dataDxfId="13">
+      <calculatedColumnFormula>ROUND(AVERAGE(C2:E2),1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{D688DEAF-FD5B-48A4-BE4D-EFF087E047F7}" name="Attendance %" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{55BCE785-43C2-4FF9-955F-B0827EAAB1A4}" name="Academic Status" dataDxfId="12">
+    <tableColumn id="7" xr3:uid="{D688DEAF-FD5B-48A4-BE4D-EFF087E047F7}" name="Attendance %" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{55BCE785-43C2-4FF9-955F-B0827EAAB1A4}" name="Academic Status" dataDxfId="11">
       <calculatedColumnFormula>IF(F2&lt;60,"FAIL","PASS")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{27EF9F5C-E441-4681-ABDD-B1B9B022F347}" name="Attendance Status" dataDxfId="11">
+    <tableColumn id="9" xr3:uid="{27EF9F5C-E441-4681-ABDD-B1B9B022F347}" name="Attendance Status" dataDxfId="10">
       <calculatedColumnFormula>IF(G2&lt;75,"FAIL","PASS")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{7633FCD6-5A02-4E88-BA52-98424D0C0C8F}" name="Risk Category" dataDxfId="10">
+    <tableColumn id="10" xr3:uid="{7633FCD6-5A02-4E88-BA52-98424D0C0C8F}" name="Risk Category" dataDxfId="9">
       <calculatedColumnFormula>IF(AND(H2="FAIL",I2="FAIL"),"RED - Dual Risk",IF(OR(H2="FAIL",I2="FAIL"),"YELLOW - Single Risk","GREEN - Satisfactory"))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="11" xr3:uid="{0E14D914-40DA-43FA-B564-1F3C424BD4F3}" name="Column1"/>
-    <tableColumn id="12" xr3:uid="{3578749C-4592-42E8-84C6-9EC16263B5C2}" name="Attn (Green)" dataDxfId="9">
+    <tableColumn id="12" xr3:uid="{3578749C-4592-42E8-84C6-9EC16263B5C2}" name="Attn (Green)" dataDxfId="8">
       <calculatedColumnFormula>IF(J2="GREEN - Satisfactory",G2,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{97F6FB84-6DB3-4CDC-9365-7888C7F0968C}" name="Avg (Green)" dataDxfId="8">
+    <tableColumn id="13" xr3:uid="{97F6FB84-6DB3-4CDC-9365-7888C7F0968C}" name="Avg (Green)" dataDxfId="7">
       <calculatedColumnFormula>IF(J2="GREEN - Satisfactory",F2,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{05BB641D-45A0-4F05-BD91-5406B37466CE}" name="Attn (Yellow)" dataDxfId="7">
+    <tableColumn id="14" xr3:uid="{05BB641D-45A0-4F05-BD91-5406B37466CE}" name="Attn (Yellow)" dataDxfId="6">
       <calculatedColumnFormula>IF(J2="YELLOW - Single Risk",G2,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{032CED30-8FFB-4376-91FF-E90F54F13E50}" name="Avg (Yellow)" dataDxfId="6">
+    <tableColumn id="15" xr3:uid="{032CED30-8FFB-4376-91FF-E90F54F13E50}" name="Avg (Yellow)" dataDxfId="5">
       <calculatedColumnFormula>IF(J2="YELLOW - Single Risk",F2,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{3EF7A40C-BE44-4B68-A24F-682FBB3D12BF}" name="Attn (Red)" dataDxfId="5">
+    <tableColumn id="16" xr3:uid="{3EF7A40C-BE44-4B68-A24F-682FBB3D12BF}" name="Attn (Red)" dataDxfId="4">
       <calculatedColumnFormula>IF(J2="RED - Dual Risk",G2,"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{57EA4195-FC04-499D-BC5C-3B4EF5EB6998}" name="Avg (Red)" dataDxfId="4">
+    <tableColumn id="17" xr3:uid="{57EA4195-FC04-499D-BC5C-3B4EF5EB6998}" name="Avg (Red)" dataDxfId="3">
       <calculatedColumnFormula>IF(J2="RED - Dual Risk",F2,"")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="18" xr3:uid="{A8C80ED2-5B3E-4C33-8FCC-0EF99047177E}" name="AttnLine_X"/>
@@ -4390,90 +4402,90 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:U43"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="6" width="11.5546875" customWidth="1"/>
+    <col min="3" max="6" width="11.5" customWidth="1"/>
     <col min="7" max="7" width="13" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="16" customWidth="1"/>
     <col min="10" max="10" width="20" customWidth="1"/>
-    <col min="11" max="11" width="11.44140625" customWidth="1"/>
-    <col min="12" max="21" width="11.109375" customWidth="1"/>
+    <col min="11" max="11" width="11.5" customWidth="1"/>
+    <col min="12" max="21" width="11.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="C1" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="E1" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="F1" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="G1" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="H1" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="H1" s="16" t="s">
+      <c r="I1" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="J1" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="J1" s="16" t="s">
+      <c r="K1" t="s">
+        <v>115</v>
+      </c>
+      <c r="L1" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="K1" t="s">
-        <v>159</v>
-      </c>
-      <c r="L1" s="17" t="s">
+      <c r="M1" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="M1" s="17" t="s">
+      <c r="N1" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="N1" s="17" t="s">
+      <c r="O1" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="O1" s="17" t="s">
+      <c r="P1" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="P1" s="17" t="s">
+      <c r="Q1" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="Q1" s="17" t="s">
+      <c r="R1" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="R1" s="17" t="s">
+      <c r="S1" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="S1" s="17" t="s">
+      <c r="T1" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="T1" s="17" t="s">
+      <c r="U1" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="U1" s="17" t="s">
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A2" s="9" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>60</v>
+      <c r="B2" s="26" t="s">
+        <v>117</v>
       </c>
       <c r="C2" s="9">
         <v>46</v>
@@ -4485,8 +4497,8 @@
         <v>54</v>
       </c>
       <c r="F2" s="18">
-        <f t="shared" ref="F2:F41" si="0">AVERAGE(C2:E2)</f>
-        <v>48.666666666666664</v>
+        <f t="shared" ref="F2:F41" si="0">ROUND(AVERAGE(C2:E2),1)</f>
+        <v>48.7</v>
       </c>
       <c r="G2" s="19">
         <v>56.3</v>
@@ -4525,7 +4537,7 @@
       </c>
       <c r="Q2" s="22">
         <f t="shared" ref="Q2:Q41" si="9">IF(J2="RED - Dual Risk",F2,"")</f>
-        <v>48.666666666666664</v>
+        <v>48.7</v>
       </c>
       <c r="R2">
         <v>0</v>
@@ -4540,12 +4552,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>62</v>
+        <v>59</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>118</v>
       </c>
       <c r="C3" s="9">
         <v>36</v>
@@ -4558,7 +4570,7 @@
       </c>
       <c r="F3" s="18">
         <f t="shared" si="0"/>
-        <v>47.666666666666664</v>
+        <v>47.7</v>
       </c>
       <c r="G3" s="19">
         <v>62.9</v>
@@ -4597,7 +4609,7 @@
       </c>
       <c r="Q3" s="22">
         <f t="shared" si="9"/>
-        <v>47.666666666666664</v>
+        <v>47.7</v>
       </c>
       <c r="R3">
         <v>100</v>
@@ -4612,12 +4624,12 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>64</v>
+        <v>60</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>119</v>
       </c>
       <c r="C4" s="9">
         <v>52</v>
@@ -4630,7 +4642,7 @@
       </c>
       <c r="F4" s="18">
         <f t="shared" si="0"/>
-        <v>50.333333333333336</v>
+        <v>50.3</v>
       </c>
       <c r="G4" s="19">
         <v>82.4</v>
@@ -4661,7 +4673,7 @@
       </c>
       <c r="O4" s="22">
         <f t="shared" si="7"/>
-        <v>50.333333333333336</v>
+        <v>50.3</v>
       </c>
       <c r="P4" s="20" t="str">
         <f t="shared" si="8"/>
@@ -4672,12 +4684,12 @@
         <v/>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>66</v>
+        <v>61</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>120</v>
       </c>
       <c r="C5" s="9">
         <v>84</v>
@@ -4690,7 +4702,7 @@
       </c>
       <c r="F5" s="18">
         <f t="shared" si="0"/>
-        <v>84.666666666666671</v>
+        <v>84.7</v>
       </c>
       <c r="G5" s="19">
         <v>92.2</v>
@@ -4713,7 +4725,7 @@
       </c>
       <c r="M5" s="22">
         <f t="shared" si="5"/>
-        <v>84.666666666666671</v>
+        <v>84.7</v>
       </c>
       <c r="N5" s="20" t="str">
         <f t="shared" si="6"/>
@@ -4732,12 +4744,12 @@
         <v/>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>68</v>
+        <v>62</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>121</v>
       </c>
       <c r="C6" s="9">
         <v>63</v>
@@ -4750,7 +4762,7 @@
       </c>
       <c r="F6" s="18">
         <f t="shared" si="0"/>
-        <v>72.333333333333329</v>
+        <v>72.3</v>
       </c>
       <c r="G6" s="19">
         <v>73.599999999999994</v>
@@ -4781,7 +4793,7 @@
       </c>
       <c r="O6" s="22">
         <f t="shared" si="7"/>
-        <v>72.333333333333329</v>
+        <v>72.3</v>
       </c>
       <c r="P6" s="20" t="str">
         <f t="shared" si="8"/>
@@ -4792,12 +4804,12 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>70</v>
+        <v>63</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>122</v>
       </c>
       <c r="C7" s="9">
         <v>75</v>
@@ -4810,7 +4822,7 @@
       </c>
       <c r="F7" s="18">
         <f t="shared" si="0"/>
-        <v>75.666666666666671</v>
+        <v>75.7</v>
       </c>
       <c r="G7" s="19">
         <v>56.7</v>
@@ -4841,7 +4853,7 @@
       </c>
       <c r="O7" s="22">
         <f t="shared" si="7"/>
-        <v>75.666666666666671</v>
+        <v>75.7</v>
       </c>
       <c r="P7" s="20" t="str">
         <f t="shared" si="8"/>
@@ -4852,12 +4864,12 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>72</v>
+        <v>64</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>123</v>
       </c>
       <c r="C8" s="9">
         <v>84</v>
@@ -4870,7 +4882,7 @@
       </c>
       <c r="F8" s="18">
         <f t="shared" si="0"/>
-        <v>79.666666666666671</v>
+        <v>79.7</v>
       </c>
       <c r="G8" s="19">
         <v>84.2</v>
@@ -4893,7 +4905,7 @@
       </c>
       <c r="M8" s="22">
         <f t="shared" si="5"/>
-        <v>79.666666666666671</v>
+        <v>79.7</v>
       </c>
       <c r="N8" s="20" t="str">
         <f t="shared" si="6"/>
@@ -4912,12 +4924,12 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>74</v>
+        <v>65</v>
+      </c>
+      <c r="B9" s="26" t="s">
+        <v>124</v>
       </c>
       <c r="C9" s="9">
         <v>48</v>
@@ -4930,7 +4942,7 @@
       </c>
       <c r="F9" s="18">
         <f t="shared" si="0"/>
-        <v>49.666666666666664</v>
+        <v>49.7</v>
       </c>
       <c r="G9" s="19">
         <v>90</v>
@@ -4961,7 +4973,7 @@
       </c>
       <c r="O9" s="22">
         <f t="shared" si="7"/>
-        <v>49.666666666666664</v>
+        <v>49.7</v>
       </c>
       <c r="P9" s="20" t="str">
         <f t="shared" si="8"/>
@@ -4972,12 +4984,12 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>76</v>
+        <v>66</v>
+      </c>
+      <c r="B10" s="26" t="s">
+        <v>125</v>
       </c>
       <c r="C10" s="9">
         <v>52</v>
@@ -4990,7 +5002,7 @@
       </c>
       <c r="F10" s="18">
         <f t="shared" si="0"/>
-        <v>50.666666666666664</v>
+        <v>50.7</v>
       </c>
       <c r="G10" s="19">
         <v>53.9</v>
@@ -5029,15 +5041,15 @@
       </c>
       <c r="Q10" s="22">
         <f t="shared" si="9"/>
-        <v>50.666666666666664</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+        <v>50.7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>78</v>
+        <v>67</v>
+      </c>
+      <c r="B11" s="26" t="s">
+        <v>126</v>
       </c>
       <c r="C11" s="9">
         <v>85</v>
@@ -5050,7 +5062,7 @@
       </c>
       <c r="F11" s="18">
         <f t="shared" si="0"/>
-        <v>86.333333333333329</v>
+        <v>86.3</v>
       </c>
       <c r="G11" s="19">
         <v>81.099999999999994</v>
@@ -5073,7 +5085,7 @@
       </c>
       <c r="M11" s="22">
         <f t="shared" si="5"/>
-        <v>86.333333333333329</v>
+        <v>86.3</v>
       </c>
       <c r="N11" s="20" t="str">
         <f t="shared" si="6"/>
@@ -5092,12 +5104,12 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>80</v>
+        <v>68</v>
+      </c>
+      <c r="B12" s="26" t="s">
+        <v>127</v>
       </c>
       <c r="C12" s="9">
         <v>81</v>
@@ -5110,7 +5122,7 @@
       </c>
       <c r="F12" s="18">
         <f t="shared" si="0"/>
-        <v>73.333333333333329</v>
+        <v>73.3</v>
       </c>
       <c r="G12" s="19">
         <v>69.7</v>
@@ -5141,7 +5153,7 @@
       </c>
       <c r="O12" s="22">
         <f t="shared" si="7"/>
-        <v>73.333333333333329</v>
+        <v>73.3</v>
       </c>
       <c r="P12" s="20" t="str">
         <f t="shared" si="8"/>
@@ -5152,12 +5164,12 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>82</v>
+        <v>69</v>
+      </c>
+      <c r="B13" s="26" t="s">
+        <v>128</v>
       </c>
       <c r="C13" s="9">
         <v>81</v>
@@ -5170,7 +5182,7 @@
       </c>
       <c r="F13" s="18">
         <f t="shared" si="0"/>
-        <v>81.666666666666671</v>
+        <v>81.7</v>
       </c>
       <c r="G13" s="19">
         <v>51.6</v>
@@ -5201,7 +5213,7 @@
       </c>
       <c r="O13" s="22">
         <f t="shared" si="7"/>
-        <v>81.666666666666671</v>
+        <v>81.7</v>
       </c>
       <c r="P13" s="20" t="str">
         <f t="shared" si="8"/>
@@ -5212,12 +5224,12 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>84</v>
+        <v>70</v>
+      </c>
+      <c r="B14" s="26" t="s">
+        <v>129</v>
       </c>
       <c r="C14" s="9">
         <v>81</v>
@@ -5230,7 +5242,7 @@
       </c>
       <c r="F14" s="18">
         <f t="shared" si="0"/>
-        <v>82.333333333333329</v>
+        <v>82.3</v>
       </c>
       <c r="G14" s="19">
         <v>59.5</v>
@@ -5261,7 +5273,7 @@
       </c>
       <c r="O14" s="22">
         <f t="shared" si="7"/>
-        <v>82.333333333333329</v>
+        <v>82.3</v>
       </c>
       <c r="P14" s="20" t="str">
         <f t="shared" si="8"/>
@@ -5272,12 +5284,12 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>86</v>
+        <v>71</v>
+      </c>
+      <c r="B15" s="26" t="s">
+        <v>130</v>
       </c>
       <c r="C15" s="9">
         <v>54</v>
@@ -5290,7 +5302,7 @@
       </c>
       <c r="F15" s="18">
         <f t="shared" si="0"/>
-        <v>48.666666666666664</v>
+        <v>48.7</v>
       </c>
       <c r="G15" s="19">
         <v>79.099999999999994</v>
@@ -5321,7 +5333,7 @@
       </c>
       <c r="O15" s="22">
         <f t="shared" si="7"/>
-        <v>48.666666666666664</v>
+        <v>48.7</v>
       </c>
       <c r="P15" s="20" t="str">
         <f t="shared" si="8"/>
@@ -5332,12 +5344,12 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>88</v>
+        <v>72</v>
+      </c>
+      <c r="B16" s="26" t="s">
+        <v>131</v>
       </c>
       <c r="C16" s="9">
         <v>57</v>
@@ -5392,12 +5404,12 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A17" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>90</v>
+        <v>73</v>
+      </c>
+      <c r="B17" s="26" t="s">
+        <v>132</v>
       </c>
       <c r="C17" s="9">
         <v>88</v>
@@ -5410,7 +5422,7 @@
       </c>
       <c r="F17" s="18">
         <f t="shared" si="0"/>
-        <v>90.666666666666671</v>
+        <v>90.7</v>
       </c>
       <c r="G17" s="19">
         <v>84.3</v>
@@ -5433,7 +5445,7 @@
       </c>
       <c r="M17" s="22">
         <f t="shared" si="5"/>
-        <v>90.666666666666671</v>
+        <v>90.7</v>
       </c>
       <c r="N17" s="20" t="str">
         <f t="shared" si="6"/>
@@ -5452,12 +5464,12 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>92</v>
+        <v>74</v>
+      </c>
+      <c r="B18" s="26" t="s">
+        <v>133</v>
       </c>
       <c r="C18" s="9">
         <v>69</v>
@@ -5470,7 +5482,7 @@
       </c>
       <c r="F18" s="18">
         <f t="shared" si="0"/>
-        <v>84.666666666666671</v>
+        <v>84.7</v>
       </c>
       <c r="G18" s="19">
         <v>78.099999999999994</v>
@@ -5493,7 +5505,7 @@
       </c>
       <c r="M18" s="22">
         <f t="shared" si="5"/>
-        <v>84.666666666666671</v>
+        <v>84.7</v>
       </c>
       <c r="N18" s="20" t="str">
         <f t="shared" si="6"/>
@@ -5512,12 +5524,12 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>94</v>
+        <v>75</v>
+      </c>
+      <c r="B19" s="26" t="s">
+        <v>134</v>
       </c>
       <c r="C19" s="9">
         <v>64</v>
@@ -5530,7 +5542,7 @@
       </c>
       <c r="F19" s="18">
         <f t="shared" si="0"/>
-        <v>67.333333333333329</v>
+        <v>67.3</v>
       </c>
       <c r="G19" s="19">
         <v>65.099999999999994</v>
@@ -5561,7 +5573,7 @@
       </c>
       <c r="O19" s="22">
         <f t="shared" si="7"/>
-        <v>67.333333333333329</v>
+        <v>67.3</v>
       </c>
       <c r="P19" s="20" t="str">
         <f t="shared" si="8"/>
@@ -5572,12 +5584,12 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A20" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>96</v>
+        <v>76</v>
+      </c>
+      <c r="B20" s="26" t="s">
+        <v>135</v>
       </c>
       <c r="C20" s="9">
         <v>53</v>
@@ -5590,7 +5602,7 @@
       </c>
       <c r="F20" s="18">
         <f t="shared" si="0"/>
-        <v>51.333333333333336</v>
+        <v>51.3</v>
       </c>
       <c r="G20" s="19">
         <v>84.5</v>
@@ -5621,7 +5633,7 @@
       </c>
       <c r="O20" s="22">
         <f t="shared" si="7"/>
-        <v>51.333333333333336</v>
+        <v>51.3</v>
       </c>
       <c r="P20" s="20" t="str">
         <f t="shared" si="8"/>
@@ -5632,12 +5644,12 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A21" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>98</v>
+        <v>77</v>
+      </c>
+      <c r="B21" s="26" t="s">
+        <v>136</v>
       </c>
       <c r="C21" s="9">
         <v>90</v>
@@ -5692,12 +5704,12 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A22" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>100</v>
+        <v>78</v>
+      </c>
+      <c r="B22" s="26" t="s">
+        <v>137</v>
       </c>
       <c r="C22" s="9">
         <v>61</v>
@@ -5710,7 +5722,7 @@
       </c>
       <c r="F22" s="18">
         <f t="shared" si="0"/>
-        <v>74.666666666666671</v>
+        <v>74.7</v>
       </c>
       <c r="G22" s="19">
         <v>68</v>
@@ -5741,7 +5753,7 @@
       </c>
       <c r="O22" s="22">
         <f t="shared" si="7"/>
-        <v>74.666666666666671</v>
+        <v>74.7</v>
       </c>
       <c r="P22" s="20" t="str">
         <f t="shared" si="8"/>
@@ -5752,12 +5764,12 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>102</v>
+        <v>79</v>
+      </c>
+      <c r="B23" s="26" t="s">
+        <v>138</v>
       </c>
       <c r="C23" s="9">
         <v>82</v>
@@ -5770,7 +5782,7 @@
       </c>
       <c r="F23" s="18">
         <f t="shared" si="0"/>
-        <v>76.333333333333329</v>
+        <v>76.3</v>
       </c>
       <c r="G23" s="19">
         <v>86</v>
@@ -5793,7 +5805,7 @@
       </c>
       <c r="M23" s="22">
         <f t="shared" si="5"/>
-        <v>76.333333333333329</v>
+        <v>76.3</v>
       </c>
       <c r="N23" s="20" t="str">
         <f t="shared" si="6"/>
@@ -5812,12 +5824,12 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A24" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>104</v>
+        <v>80</v>
+      </c>
+      <c r="B24" s="26" t="s">
+        <v>139</v>
       </c>
       <c r="C24" s="9">
         <v>90</v>
@@ -5872,12 +5884,12 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>106</v>
+        <v>81</v>
+      </c>
+      <c r="B25" s="26" t="s">
+        <v>140</v>
       </c>
       <c r="C25" s="9">
         <v>72</v>
@@ -5890,7 +5902,7 @@
       </c>
       <c r="F25" s="18">
         <f t="shared" si="0"/>
-        <v>77.333333333333329</v>
+        <v>77.3</v>
       </c>
       <c r="G25" s="19">
         <v>70.900000000000006</v>
@@ -5921,7 +5933,7 @@
       </c>
       <c r="O25" s="22">
         <f t="shared" si="7"/>
-        <v>77.333333333333329</v>
+        <v>77.3</v>
       </c>
       <c r="P25" s="20" t="str">
         <f t="shared" si="8"/>
@@ -5932,12 +5944,12 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A26" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>108</v>
+        <v>82</v>
+      </c>
+      <c r="B26" s="26" t="s">
+        <v>141</v>
       </c>
       <c r="C26" s="9">
         <v>49</v>
@@ -5950,7 +5962,7 @@
       </c>
       <c r="F26" s="18">
         <f t="shared" si="0"/>
-        <v>54.666666666666664</v>
+        <v>54.7</v>
       </c>
       <c r="G26" s="19">
         <v>80.400000000000006</v>
@@ -5981,7 +5993,7 @@
       </c>
       <c r="O26" s="22">
         <f t="shared" si="7"/>
-        <v>54.666666666666664</v>
+        <v>54.7</v>
       </c>
       <c r="P26" s="20" t="str">
         <f t="shared" si="8"/>
@@ -5992,12 +6004,12 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A27" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>110</v>
+        <v>83</v>
+      </c>
+      <c r="B27" s="26" t="s">
+        <v>142</v>
       </c>
       <c r="C27" s="9">
         <v>51</v>
@@ -6052,12 +6064,12 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A28" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>112</v>
+        <v>84</v>
+      </c>
+      <c r="B28" s="26" t="s">
+        <v>143</v>
       </c>
       <c r="C28" s="9">
         <v>94</v>
@@ -6070,7 +6082,7 @@
       </c>
       <c r="F28" s="18">
         <f t="shared" si="0"/>
-        <v>78.666666666666671</v>
+        <v>78.7</v>
       </c>
       <c r="G28" s="19">
         <v>87.2</v>
@@ -6093,7 +6105,7 @@
       </c>
       <c r="M28" s="22">
         <f t="shared" si="5"/>
-        <v>78.666666666666671</v>
+        <v>78.7</v>
       </c>
       <c r="N28" s="20" t="str">
         <f t="shared" si="6"/>
@@ -6112,12 +6124,12 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A29" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>114</v>
+        <v>85</v>
+      </c>
+      <c r="B29" s="26" t="s">
+        <v>144</v>
       </c>
       <c r="C29" s="9">
         <v>68</v>
@@ -6130,7 +6142,7 @@
       </c>
       <c r="F29" s="18">
         <f t="shared" si="0"/>
-        <v>77.333333333333329</v>
+        <v>77.3</v>
       </c>
       <c r="G29" s="19">
         <v>81.5</v>
@@ -6153,7 +6165,7 @@
       </c>
       <c r="M29" s="22">
         <f t="shared" si="5"/>
-        <v>77.333333333333329</v>
+        <v>77.3</v>
       </c>
       <c r="N29" s="20" t="str">
         <f t="shared" si="6"/>
@@ -6172,12 +6184,12 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A30" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>116</v>
+        <v>86</v>
+      </c>
+      <c r="B30" s="26" t="s">
+        <v>145</v>
       </c>
       <c r="C30" s="9">
         <v>42</v>
@@ -6232,12 +6244,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A31" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>118</v>
+        <v>87</v>
+      </c>
+      <c r="B31" s="26" t="s">
+        <v>146</v>
       </c>
       <c r="C31" s="9">
         <v>50</v>
@@ -6250,7 +6262,7 @@
       </c>
       <c r="F31" s="18">
         <f t="shared" si="0"/>
-        <v>46.333333333333336</v>
+        <v>46.3</v>
       </c>
       <c r="G31" s="19">
         <v>68.400000000000006</v>
@@ -6289,15 +6301,15 @@
       </c>
       <c r="Q31" s="22">
         <f t="shared" si="9"/>
-        <v>46.333333333333336</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
+        <v>46.3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A32" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>120</v>
+        <v>88</v>
+      </c>
+      <c r="B32" s="26" t="s">
+        <v>147</v>
       </c>
       <c r="C32" s="9">
         <v>69</v>
@@ -6310,7 +6322,7 @@
       </c>
       <c r="F32" s="18">
         <f t="shared" si="0"/>
-        <v>85.333333333333329</v>
+        <v>85.3</v>
       </c>
       <c r="G32" s="19">
         <v>79.8</v>
@@ -6333,7 +6345,7 @@
       </c>
       <c r="M32" s="22">
         <f t="shared" si="5"/>
-        <v>85.333333333333329</v>
+        <v>85.3</v>
       </c>
       <c r="N32" s="20" t="str">
         <f t="shared" si="6"/>
@@ -6352,12 +6364,12 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A33" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="B33" s="9" t="s">
-        <v>122</v>
+        <v>89</v>
+      </c>
+      <c r="B33" s="26" t="s">
+        <v>148</v>
       </c>
       <c r="C33" s="9">
         <v>94</v>
@@ -6370,7 +6382,7 @@
       </c>
       <c r="F33" s="18">
         <f t="shared" si="0"/>
-        <v>85.333333333333329</v>
+        <v>85.3</v>
       </c>
       <c r="G33" s="19">
         <v>72.3</v>
@@ -6401,7 +6413,7 @@
       </c>
       <c r="O33" s="22">
         <f t="shared" si="7"/>
-        <v>85.333333333333329</v>
+        <v>85.3</v>
       </c>
       <c r="P33" s="20" t="str">
         <f t="shared" si="8"/>
@@ -6412,12 +6424,12 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A34" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="B34" s="9" t="s">
-        <v>124</v>
+        <v>90</v>
+      </c>
+      <c r="B34" s="26" t="s">
+        <v>149</v>
       </c>
       <c r="C34" s="9">
         <v>58</v>
@@ -6472,12 +6484,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A35" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="B35" s="9" t="s">
-        <v>126</v>
+        <v>91</v>
+      </c>
+      <c r="B35" s="26" t="s">
+        <v>150</v>
       </c>
       <c r="C35" s="9">
         <v>47</v>
@@ -6490,7 +6502,7 @@
       </c>
       <c r="F35" s="18">
         <f t="shared" si="0"/>
-        <v>52.666666666666664</v>
+        <v>52.7</v>
       </c>
       <c r="G35" s="19">
         <v>59</v>
@@ -6529,15 +6541,15 @@
       </c>
       <c r="Q35" s="22">
         <f t="shared" si="9"/>
-        <v>52.666666666666664</v>
-      </c>
-    </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
+        <v>52.7</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A36" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="B36" s="9" t="s">
-        <v>128</v>
+        <v>92</v>
+      </c>
+      <c r="B36" s="26" t="s">
+        <v>151</v>
       </c>
       <c r="C36" s="9">
         <v>51</v>
@@ -6592,12 +6604,12 @@
         <v>46</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A37" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="B37" s="9" t="s">
-        <v>130</v>
+        <v>93</v>
+      </c>
+      <c r="B37" s="26" t="s">
+        <v>152</v>
       </c>
       <c r="C37" s="9">
         <v>42</v>
@@ -6652,12 +6664,12 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A38" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="B38" s="9" t="s">
-        <v>132</v>
+        <v>94</v>
+      </c>
+      <c r="B38" s="26" t="s">
+        <v>153</v>
       </c>
       <c r="C38" s="9">
         <v>47</v>
@@ -6670,7 +6682,7 @@
       </c>
       <c r="F38" s="18">
         <f t="shared" si="0"/>
-        <v>50.666666666666664</v>
+        <v>50.7</v>
       </c>
       <c r="G38" s="19">
         <v>76.2</v>
@@ -6701,7 +6713,7 @@
       </c>
       <c r="O38" s="22">
         <f t="shared" si="7"/>
-        <v>50.666666666666664</v>
+        <v>50.7</v>
       </c>
       <c r="P38" s="20" t="str">
         <f t="shared" si="8"/>
@@ -6712,12 +6724,12 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A39" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="B39" s="9" t="s">
-        <v>134</v>
+        <v>95</v>
+      </c>
+      <c r="B39" s="26" t="s">
+        <v>154</v>
       </c>
       <c r="C39" s="9">
         <v>41</v>
@@ -6730,7 +6742,7 @@
       </c>
       <c r="F39" s="18">
         <f t="shared" si="0"/>
-        <v>43.333333333333336</v>
+        <v>43.3</v>
       </c>
       <c r="G39" s="19">
         <v>95.9</v>
@@ -6761,7 +6773,7 @@
       </c>
       <c r="O39" s="22">
         <f t="shared" si="7"/>
-        <v>43.333333333333336</v>
+        <v>43.3</v>
       </c>
       <c r="P39" s="20" t="str">
         <f t="shared" si="8"/>
@@ -6772,12 +6784,12 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A40" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="B40" s="9" t="s">
-        <v>136</v>
+        <v>96</v>
+      </c>
+      <c r="B40" s="26" t="s">
+        <v>155</v>
       </c>
       <c r="C40" s="9">
         <v>45</v>
@@ -6790,7 +6802,7 @@
       </c>
       <c r="F40" s="18">
         <f t="shared" si="0"/>
-        <v>44.333333333333336</v>
+        <v>44.3</v>
       </c>
       <c r="G40" s="19">
         <v>55.7</v>
@@ -6829,15 +6841,15 @@
       </c>
       <c r="Q40" s="22">
         <f t="shared" si="9"/>
-        <v>44.333333333333336</v>
-      </c>
-    </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
+        <v>44.3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A41" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="B41" s="9" t="s">
-        <v>138</v>
+        <v>97</v>
+      </c>
+      <c r="B41" s="26" t="s">
+        <v>156</v>
       </c>
       <c r="C41" s="9">
         <v>56</v>
@@ -6892,12 +6904,11 @@
         <v>49</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A43" s="23" t="s">
-        <v>139</v>
-      </c>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A43" s="23"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="28" type="noConversion"/>
   <conditionalFormatting sqref="J2:J41">
     <cfRule type="expression" dxfId="2" priority="2">
       <formula>LEFT(J2,3)="RED"</formula>
@@ -6920,49 +6931,49 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.109375" customWidth="1"/>
-    <col min="2" max="12" width="10.5546875" customWidth="1"/>
+    <col min="1" max="1" width="23.1640625" customWidth="1"/>
+    <col min="2" max="12" width="10.5" customWidth="1"/>
     <col min="13" max="14" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="32" t="s">
+    <row r="1" spans="1:14" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
       <c r="N1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="33" t="s">
+    <row r="2" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="33"/>
-      <c r="C2" s="33"/>
-      <c r="D2" s="33"/>
-      <c r="E2" s="33"/>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
-      <c r="I2" s="33"/>
-      <c r="J2" s="33"/>
-      <c r="K2" s="33"/>
-      <c r="L2" s="33"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+      <c r="J2" s="28"/>
+      <c r="K2" s="28"/>
+      <c r="L2" s="28"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="M3" s="2" t="s">
         <v>3</v>
       </c>
@@ -6971,27 +6982,27 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="34" t="s">
+    <row r="4" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="35" t="s">
+      <c r="B4" s="29"/>
+      <c r="C4" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="35"/>
-      <c r="E4" s="36" t="s">
+      <c r="D4" s="30"/>
+      <c r="E4" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="36"/>
-      <c r="G4" s="37" t="s">
+      <c r="F4" s="31"/>
+      <c r="G4" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="37"/>
-      <c r="I4" s="38" t="s">
+      <c r="H4" s="32"/>
+      <c r="I4" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="J4" s="38"/>
+      <c r="J4" s="33"/>
       <c r="M4" s="2" t="s">
         <v>8</v>
       </c>
@@ -7000,32 +7011,32 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="27">
+    <row r="5" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="34">
         <f>N3</f>
         <v>40</v>
       </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="28">
+      <c r="B5" s="34"/>
+      <c r="C5" s="35">
         <f>N4</f>
         <v>10</v>
       </c>
-      <c r="D5" s="28"/>
-      <c r="E5" s="29">
+      <c r="D5" s="35"/>
+      <c r="E5" s="36">
         <f>N5</f>
         <v>20</v>
       </c>
-      <c r="F5" s="29"/>
-      <c r="G5" s="30">
+      <c r="F5" s="36"/>
+      <c r="G5" s="37">
         <f>N6</f>
         <v>10</v>
       </c>
-      <c r="H5" s="30"/>
-      <c r="I5" s="31">
+      <c r="H5" s="37"/>
+      <c r="I5" s="38">
         <f>N7</f>
         <v>0.75</v>
       </c>
-      <c r="J5" s="31"/>
+      <c r="J5" s="38"/>
       <c r="M5" s="2" t="s">
         <v>9</v>
       </c>
@@ -7034,17 +7045,17 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="27"/>
-      <c r="B6" s="27"/>
-      <c r="C6" s="28"/>
-      <c r="D6" s="28"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="30"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="31"/>
+    <row r="6" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="34"/>
+      <c r="B6" s="34"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="37"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="38"/>
+      <c r="J6" s="38"/>
       <c r="M6" s="2" t="s">
         <v>10</v>
       </c>
@@ -7053,17 +7064,17 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="27"/>
-      <c r="B7" s="27"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="29"/>
-      <c r="G7" s="30"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="31"/>
-      <c r="J7" s="31"/>
+    <row r="7" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="34"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="37"/>
+      <c r="I7" s="38"/>
+      <c r="J7" s="38"/>
       <c r="M7" s="2" t="s">
         <v>11</v>
       </c>
@@ -7072,36 +7083,36 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="26" t="s">
+    <row r="8" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26" t="s">
+      <c r="B8" s="39"/>
+      <c r="C8" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26" t="s">
+      <c r="D8" s="39"/>
+      <c r="E8" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26" t="s">
+      <c r="F8" s="39"/>
+      <c r="G8" s="39" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26" t="s">
+      <c r="H8" s="39"/>
+      <c r="I8" s="39" t="s">
         <v>13</v>
       </c>
-      <c r="J8" s="26"/>
+      <c r="J8" s="39"/>
       <c r="M8" s="2" t="s">
         <v>14</v>
       </c>
       <c r="N8" s="2">
         <f>AVERAGE('Student Data'!F2:F41)</f>
-        <v>64.39166666666668</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+        <v>64.392500000000013</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="M9" s="2" t="s">
         <v>15</v>
       </c>
@@ -7110,13 +7121,13 @@
         <v>74.362500000000011</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B10" s="4">
         <f>N8</f>
-        <v>64.39166666666668</v>
+        <v>64.392500000000013</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>17</v>
@@ -7130,7 +7141,7 @@
       </c>
       <c r="H10" s="4">
         <f>N10</f>
-        <v>43.333333333333336</v>
+        <v>43.3</v>
       </c>
       <c r="J10" s="3" t="s">
         <v>19</v>
@@ -7144,10 +7155,10 @@
       </c>
       <c r="N10" s="2">
         <f>MIN('Student Data'!F2:F41)</f>
-        <v>43.333333333333336</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+        <v>43.3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="M11" s="2" t="s">
         <v>21</v>
       </c>
@@ -7156,15 +7167,15 @@
         <v>51.6</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
         <v>23</v>
       </c>
@@ -7172,19 +7183,19 @@
         <v>24</v>
       </c>
       <c r="D14" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="F14" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="G14" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="G14" s="7" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
         <v>25</v>
       </c>
@@ -7193,7 +7204,7 @@
         <v>10</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E15" s="13">
         <v>4</v>
@@ -7205,7 +7216,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" s="10" t="s">
         <v>26</v>
       </c>
@@ -7214,7 +7225,7 @@
         <v>20</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E16" s="13">
         <v>5</v>
@@ -7226,7 +7237,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
         <v>27</v>
       </c>
@@ -7235,7 +7246,7 @@
         <v>10</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E17" s="13">
         <v>7</v>
@@ -7247,9 +7258,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D18" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E18" s="13">
         <v>9</v>
@@ -7261,9 +7272,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D19" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E19" s="13">
         <v>8</v>
@@ -7275,9 +7286,9 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D20" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E20" s="13">
         <v>6</v>
@@ -7291,6 +7302,16 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="A5:B7"/>
+    <mergeCell ref="C5:D7"/>
+    <mergeCell ref="E5:F7"/>
+    <mergeCell ref="G5:H7"/>
+    <mergeCell ref="I5:J7"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A4:B4"/>
@@ -7298,16 +7319,6 @@
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="I4:J4"/>
-    <mergeCell ref="A5:B7"/>
-    <mergeCell ref="C5:D7"/>
-    <mergeCell ref="E5:F7"/>
-    <mergeCell ref="G5:H7"/>
-    <mergeCell ref="I5:J7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="I8:J8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -7318,122 +7329,122 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A25"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="18" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="25"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="25" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="25"/>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="25" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="25" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="25"/>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" s="25" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" s="25" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" s="25" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" s="25"/>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="25" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" s="25" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" s="25" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="25"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="25" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="25" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" s="25" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" s="25" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" s="25"/>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" s="25" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" s="25" t="s">
-        <v>158</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>